<commit_message>
Ajustes pendientes fixed -  Readme Updated
</commit_message>
<xml_diff>
--- a/data/Lead_information_Formulario_Paraguay_Main.xlsx
+++ b/data/Lead_information_Formulario_Paraguay_Main.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,38 +481,38 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.chevrolet.com.py/suvs/sonic</t>
+          <t>https://www.chevrolet.com.py/solicita-una-cotizacion</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://secure-developments.com/commonwealth/paraguay/gm_forms/movs-visid?model=sonic</t>
+          <t>https://secure-developments.com/commonwealth/paraguay/gm_forms/raq</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Matías Agustín</t>
+          <t>Verónica Carolina</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Flores</t>
+          <t>Muñoz Quispe</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>58272206</t>
+          <t>41440098</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0997677958</t>
+          <t>0912230965</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>matiasagustinflores.py43@mrm.com</t>
+          <t>veronicacarolinamunozquispe_py43@mrm.com</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -520,132 +520,6 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>https://www.chevrolet.com.py/vehiculos-electricos/spark-euv/accesorios/formulario</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://secure-developments.com/commonwealth/paraguay/gm_forms/accesorios?model=spark%20euv</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Rafael Diego</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Rojas Rodriguez</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>92238907</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0956464810</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>rafaeldiegorojasrodriguez.py20@mrm.com</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>https://www.chevrolet.com.py/pickups/silverado-camioneta-pickup</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://secure-developments.com/commonwealth/paraguay/gm_forms/model-overviews?model=silverado</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Natalia</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Sanchez Campos</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>11288493</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0924662518</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nataliasanchezcampos_py88@mrm.com</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>https://www.chevrolet.com.py/solicita-una-cotizacion</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://secure-developments.com/commonwealth/paraguay/gm_forms/raq</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Verónica Carolina</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Muñoz Quispe</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>41440098</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>0912230965</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>veronicacarolinamunozquispe_py43@mrm.com</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>